<commit_message>
Added Some Missed Gems to Gem Logic - Missed that some barrels and crates in Stormy Beach are horn diveable and contain 270 gems total.
</commit_message>
<xml_diff>
--- a/worlds/spyro_aht/setup/Gem Research.xlsx
+++ b/worlds/spyro_aht/setup/Gem Research.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sean\Downloads\Archipelago Stuff\apworlds\PhoenixAP\worlds\spyro_aht\setup\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{507BE4F0-51D2-4D12-AEA8-D05DE4E99A6E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{685BD3BA-5038-49F1-A81A-A29F890C7E75}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21240" tabRatio="697" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -297,7 +297,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4189" uniqueCount="683">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4192" uniqueCount="684">
   <si>
     <t>DVEntry</t>
   </si>
@@ -2346,6 +2346,9 @@
   </si>
   <si>
     <t>[enemy] roller robot/huge robo-gnorcs/steel traps</t>
+  </si>
+  <si>
+    <t>horn diveable barrels/crates</t>
   </si>
 </sst>
 </file>
@@ -2707,7 +2710,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4BA72872-8033-4B31-8137-7B209A06634B}">
-  <dimension ref="A1:M823"/>
+  <dimension ref="A1:M824"/>
   <sheetFormatPr defaultRowHeight="28.5" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="41.140625" style="1" bestFit="1" customWidth="1"/>
@@ -2759,8 +2762,8 @@
         <v>29</v>
       </c>
       <c r="M3" s="1">
-        <f>SUM(B$2:B$1006)-M$2-M$1</f>
-        <v>424929</v>
+        <f>SUM(B$2:B$1007)-M$2-M$1</f>
+        <v>425739</v>
       </c>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.45">
@@ -2801,7 +2804,7 @@
       </c>
       <c r="M5" s="1">
         <f>M4-M3</f>
-        <v>-282105</v>
+        <v>-282915</v>
       </c>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.45">
@@ -10377,10 +10380,10 @@
         <v>307</v>
       </c>
       <c r="B551" s="1">
-        <v>325</v>
+        <v>270</v>
       </c>
       <c r="C551" s="1" t="s">
-        <v>24</v>
+        <v>683</v>
       </c>
       <c r="D551" s="3" t="s">
         <v>20</v>
@@ -10391,10 +10394,10 @@
         <v>307</v>
       </c>
       <c r="B552" s="1">
-        <v>650</v>
+        <v>325</v>
       </c>
       <c r="C552" s="1" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="D552" s="3" t="s">
         <v>20</v>
@@ -10405,13 +10408,13 @@
         <v>307</v>
       </c>
       <c r="B553" s="1">
-        <v>20</v>
+        <v>650</v>
       </c>
       <c r="C553" s="1" t="s">
-        <v>411</v>
+        <v>21</v>
       </c>
       <c r="D553" s="3" t="s">
-        <v>36</v>
+        <v>20</v>
       </c>
     </row>
     <row r="554" spans="1:4" x14ac:dyDescent="0.45">
@@ -10419,13 +10422,13 @@
         <v>307</v>
       </c>
       <c r="B554" s="1">
-        <v>180</v>
+        <v>20</v>
       </c>
       <c r="C554" s="1" t="s">
-        <v>33</v>
+        <v>411</v>
       </c>
       <c r="D554" s="3" t="s">
-        <v>20</v>
+        <v>36</v>
       </c>
     </row>
     <row r="555" spans="1:4" x14ac:dyDescent="0.45">
@@ -10433,13 +10436,13 @@
         <v>307</v>
       </c>
       <c r="B555" s="1">
-        <v>1000</v>
+        <v>180</v>
       </c>
       <c r="C555" s="1" t="s">
-        <v>308</v>
+        <v>33</v>
       </c>
       <c r="D555" s="3" t="s">
-        <v>39</v>
+        <v>20</v>
       </c>
     </row>
     <row r="556" spans="1:4" x14ac:dyDescent="0.45">
@@ -10447,13 +10450,13 @@
         <v>307</v>
       </c>
       <c r="B556" s="1">
-        <v>20</v>
+        <v>1000</v>
       </c>
       <c r="C556" s="1" t="s">
-        <v>412</v>
+        <v>308</v>
       </c>
       <c r="D556" s="3" t="s">
-        <v>48</v>
+        <v>39</v>
       </c>
     </row>
     <row r="557" spans="1:4" x14ac:dyDescent="0.45">
@@ -10464,7 +10467,7 @@
         <v>20</v>
       </c>
       <c r="C557" s="1" t="s">
-        <v>414</v>
+        <v>412</v>
       </c>
       <c r="D557" s="3" t="s">
         <v>48</v>
@@ -10478,24 +10481,24 @@
         <v>20</v>
       </c>
       <c r="C558" s="1" t="s">
-        <v>464</v>
+        <v>414</v>
       </c>
       <c r="D558" s="3" t="s">
-        <v>22</v>
+        <v>48</v>
       </c>
     </row>
     <row r="559" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A559" s="1" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
       <c r="B559" s="1">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="C559" s="1" t="s">
-        <v>412</v>
+        <v>464</v>
       </c>
       <c r="D559" s="3" t="s">
-        <v>48</v>
+        <v>22</v>
       </c>
     </row>
     <row r="560" spans="1:4" x14ac:dyDescent="0.45">
@@ -10503,32 +10506,32 @@
         <v>309</v>
       </c>
       <c r="B560" s="1">
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="C560" s="1" t="s">
-        <v>281</v>
+        <v>412</v>
       </c>
       <c r="D560" s="3" t="s">
-        <v>20</v>
+        <v>48</v>
       </c>
     </row>
     <row r="561" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A561" s="1" t="s">
-        <v>385</v>
+        <v>309</v>
+      </c>
+      <c r="B561" s="1">
+        <v>60</v>
+      </c>
+      <c r="C561" s="1" t="s">
+        <v>281</v>
+      </c>
+      <c r="D561" s="3" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="562" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A562" s="1" t="s">
-        <v>310</v>
-      </c>
-      <c r="B562" s="1">
-        <v>500</v>
-      </c>
-      <c r="C562" s="1" t="s">
-        <v>311</v>
-      </c>
-      <c r="D562" s="3" t="s">
-        <v>39</v>
+        <v>385</v>
       </c>
     </row>
     <row r="563" spans="1:4" x14ac:dyDescent="0.45">
@@ -10536,13 +10539,13 @@
         <v>310</v>
       </c>
       <c r="B563" s="1">
-        <v>50</v>
+        <v>500</v>
       </c>
       <c r="C563" s="1" t="s">
-        <v>488</v>
+        <v>311</v>
       </c>
       <c r="D563" s="3" t="s">
-        <v>395</v>
+        <v>39</v>
       </c>
     </row>
     <row r="564" spans="1:4" x14ac:dyDescent="0.45">
@@ -10553,10 +10556,10 @@
         <v>50</v>
       </c>
       <c r="C564" s="1" t="s">
-        <v>172</v>
+        <v>488</v>
       </c>
       <c r="D564" s="3" t="s">
-        <v>20</v>
+        <v>395</v>
       </c>
     </row>
     <row r="565" spans="1:4" x14ac:dyDescent="0.45">
@@ -10564,13 +10567,13 @@
         <v>310</v>
       </c>
       <c r="B565" s="1">
-        <v>1500</v>
+        <v>50</v>
       </c>
       <c r="C565" s="1" t="s">
-        <v>67</v>
+        <v>172</v>
       </c>
       <c r="D565" s="3" t="s">
-        <v>68</v>
+        <v>20</v>
       </c>
     </row>
     <row r="566" spans="1:4" x14ac:dyDescent="0.45">
@@ -10578,13 +10581,13 @@
         <v>310</v>
       </c>
       <c r="B566" s="1">
-        <v>50</v>
+        <v>1500</v>
       </c>
       <c r="C566" s="1" t="s">
-        <v>24</v>
+        <v>67</v>
       </c>
       <c r="D566" s="3" t="s">
-        <v>20</v>
+        <v>68</v>
       </c>
     </row>
     <row r="567" spans="1:4" x14ac:dyDescent="0.45">
@@ -10592,10 +10595,10 @@
         <v>310</v>
       </c>
       <c r="B567" s="1">
-        <v>25</v>
+        <v>50</v>
       </c>
       <c r="C567" s="1" t="s">
-        <v>57</v>
+        <v>24</v>
       </c>
       <c r="D567" s="3" t="s">
         <v>20</v>
@@ -10606,10 +10609,10 @@
         <v>310</v>
       </c>
       <c r="B568" s="1">
-        <v>447</v>
+        <v>25</v>
       </c>
       <c r="C568" s="1" t="s">
-        <v>19</v>
+        <v>57</v>
       </c>
       <c r="D568" s="3" t="s">
         <v>20</v>
@@ -10617,10 +10620,10 @@
     </row>
     <row r="569" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A569" s="1" t="s">
-        <v>312</v>
+        <v>310</v>
       </c>
       <c r="B569" s="1">
-        <v>131</v>
+        <v>447</v>
       </c>
       <c r="C569" s="1" t="s">
         <v>19</v>
@@ -10634,13 +10637,13 @@
         <v>312</v>
       </c>
       <c r="B570" s="1">
-        <v>50</v>
+        <v>131</v>
       </c>
       <c r="C570" s="1" t="s">
-        <v>492</v>
+        <v>19</v>
       </c>
       <c r="D570" s="3" t="s">
-        <v>388</v>
+        <v>20</v>
       </c>
     </row>
     <row r="571" spans="1:4" x14ac:dyDescent="0.45">
@@ -10648,13 +10651,13 @@
         <v>312</v>
       </c>
       <c r="B571" s="1">
-        <v>25</v>
+        <v>50</v>
       </c>
       <c r="C571" s="1" t="s">
-        <v>257</v>
+        <v>492</v>
       </c>
       <c r="D571" s="3" t="s">
-        <v>39</v>
+        <v>388</v>
       </c>
     </row>
     <row r="572" spans="1:4" x14ac:dyDescent="0.45">
@@ -10662,13 +10665,13 @@
         <v>312</v>
       </c>
       <c r="B572" s="1">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="C572" s="1" t="s">
-        <v>493</v>
+        <v>257</v>
       </c>
       <c r="D572" s="3" t="s">
-        <v>388</v>
+        <v>39</v>
       </c>
     </row>
     <row r="573" spans="1:4" x14ac:dyDescent="0.45">
@@ -10676,24 +10679,24 @@
         <v>312</v>
       </c>
       <c r="B573" s="1">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="C573" s="1" t="s">
-        <v>240</v>
+        <v>493</v>
       </c>
       <c r="D573" s="3" t="s">
-        <v>20</v>
+        <v>388</v>
       </c>
     </row>
     <row r="574" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A574" s="1" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="B574" s="1">
-        <v>610</v>
+        <v>30</v>
       </c>
       <c r="C574" s="1" t="s">
-        <v>19</v>
+        <v>240</v>
       </c>
       <c r="D574" s="3" t="s">
         <v>20</v>
@@ -10704,13 +10707,13 @@
         <v>313</v>
       </c>
       <c r="B575" s="1">
-        <v>25</v>
+        <v>610</v>
       </c>
       <c r="C575" s="1" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="D575" s="3" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
     </row>
     <row r="576" spans="1:4" x14ac:dyDescent="0.45">
@@ -10718,13 +10721,13 @@
         <v>313</v>
       </c>
       <c r="B576" s="1">
-        <v>150</v>
+        <v>25</v>
       </c>
       <c r="C576" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D576" s="3" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="577" spans="1:4" x14ac:dyDescent="0.45">
@@ -10732,13 +10735,13 @@
         <v>313</v>
       </c>
       <c r="B577" s="1">
-        <v>100</v>
+        <v>150</v>
       </c>
       <c r="C577" s="1" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="D577" s="3" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="578" spans="1:4" x14ac:dyDescent="0.45">
@@ -10746,13 +10749,13 @@
         <v>313</v>
       </c>
       <c r="B578" s="1">
-        <v>400</v>
+        <v>100</v>
       </c>
       <c r="C578" s="1" t="s">
-        <v>494</v>
+        <v>21</v>
       </c>
       <c r="D578" s="3" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
     </row>
     <row r="579" spans="1:4" x14ac:dyDescent="0.45">
@@ -10760,27 +10763,27 @@
         <v>313</v>
       </c>
       <c r="B579" s="1">
-        <v>30</v>
+        <v>400</v>
       </c>
       <c r="C579" s="1" t="s">
-        <v>33</v>
+        <v>494</v>
       </c>
       <c r="D579" s="3" t="s">
-        <v>35</v>
+        <v>22</v>
       </c>
     </row>
     <row r="580" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A580" s="1" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="B580" s="1">
-        <v>225</v>
+        <v>30</v>
       </c>
       <c r="C580" s="1" t="s">
-        <v>493</v>
+        <v>33</v>
       </c>
       <c r="D580" s="3" t="s">
-        <v>20</v>
+        <v>35</v>
       </c>
     </row>
     <row r="581" spans="1:4" x14ac:dyDescent="0.45">
@@ -10788,10 +10791,10 @@
         <v>314</v>
       </c>
       <c r="B581" s="1">
-        <v>443</v>
+        <v>225</v>
       </c>
       <c r="C581" s="1" t="s">
-        <v>662</v>
+        <v>493</v>
       </c>
       <c r="D581" s="3" t="s">
         <v>20</v>
@@ -10805,7 +10808,7 @@
         <v>443</v>
       </c>
       <c r="C582" s="1" t="s">
-        <v>663</v>
+        <v>662</v>
       </c>
       <c r="D582" s="3" t="s">
         <v>20</v>
@@ -10813,13 +10816,13 @@
     </row>
     <row r="583" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A583" s="1" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="B583" s="1">
-        <v>50</v>
+        <v>443</v>
       </c>
       <c r="C583" s="1" t="s">
-        <v>672</v>
+        <v>663</v>
       </c>
       <c r="D583" s="3" t="s">
         <v>20</v>
@@ -10830,13 +10833,13 @@
         <v>315</v>
       </c>
       <c r="B584" s="1">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="C584" s="1" t="s">
-        <v>411</v>
+        <v>672</v>
       </c>
       <c r="D584" s="3" t="s">
-        <v>36</v>
+        <v>20</v>
       </c>
     </row>
     <row r="585" spans="1:4" x14ac:dyDescent="0.45">
@@ -10844,13 +10847,13 @@
         <v>315</v>
       </c>
       <c r="B585" s="1">
-        <v>153</v>
+        <v>40</v>
       </c>
       <c r="C585" s="1" t="s">
-        <v>19</v>
+        <v>411</v>
       </c>
       <c r="D585" s="3" t="s">
-        <v>20</v>
+        <v>36</v>
       </c>
     </row>
     <row r="586" spans="1:4" x14ac:dyDescent="0.45">
@@ -10858,13 +10861,13 @@
         <v>315</v>
       </c>
       <c r="B586" s="1">
-        <v>20</v>
+        <v>153</v>
       </c>
       <c r="C586" s="1" t="s">
-        <v>413</v>
+        <v>19</v>
       </c>
       <c r="D586" s="3" t="s">
-        <v>47</v>
+        <v>20</v>
       </c>
     </row>
     <row r="587" spans="1:4" x14ac:dyDescent="0.45">
@@ -10875,10 +10878,10 @@
         <v>20</v>
       </c>
       <c r="C587" s="1" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="D587" s="3" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="588" spans="1:4" x14ac:dyDescent="0.45">
@@ -10886,13 +10889,13 @@
         <v>315</v>
       </c>
       <c r="B588" s="1">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="C588" s="1" t="s">
-        <v>23</v>
+        <v>414</v>
       </c>
       <c r="D588" s="3" t="s">
-        <v>26</v>
+        <v>48</v>
       </c>
     </row>
     <row r="589" spans="1:4" x14ac:dyDescent="0.45">
@@ -10900,41 +10903,41 @@
         <v>315</v>
       </c>
       <c r="B589" s="1">
-        <v>25</v>
+        <v>50</v>
       </c>
       <c r="C589" s="1" t="s">
-        <v>236</v>
+        <v>23</v>
       </c>
       <c r="D589" s="3" t="s">
-        <v>35</v>
+        <v>26</v>
       </c>
     </row>
     <row r="590" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A590" s="1" t="s">
-        <v>674</v>
+        <v>315</v>
       </c>
       <c r="B590" s="1">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="C590" s="1" t="s">
-        <v>673</v>
+        <v>236</v>
       </c>
       <c r="D590" s="3" t="s">
-        <v>20</v>
+        <v>35</v>
       </c>
     </row>
     <row r="591" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A591" s="1" t="s">
-        <v>675</v>
+        <v>674</v>
       </c>
       <c r="B591" s="1">
-        <v>25</v>
+        <v>50</v>
       </c>
       <c r="C591" s="1" t="s">
-        <v>389</v>
+        <v>673</v>
       </c>
       <c r="D591" s="3" t="s">
-        <v>47</v>
+        <v>20</v>
       </c>
     </row>
     <row r="592" spans="1:4" x14ac:dyDescent="0.45">
@@ -10942,13 +10945,13 @@
         <v>675</v>
       </c>
       <c r="B592" s="1">
-        <v>130</v>
+        <v>25</v>
       </c>
       <c r="C592" s="1" t="s">
-        <v>19</v>
+        <v>389</v>
       </c>
       <c r="D592" s="3" t="s">
-        <v>20</v>
+        <v>47</v>
       </c>
     </row>
     <row r="593" spans="1:4" x14ac:dyDescent="0.45">
@@ -10956,10 +10959,10 @@
         <v>675</v>
       </c>
       <c r="B593" s="1">
-        <v>55</v>
+        <v>130</v>
       </c>
       <c r="C593" s="1" t="s">
-        <v>229</v>
+        <v>19</v>
       </c>
       <c r="D593" s="3" t="s">
         <v>20</v>
@@ -10970,10 +10973,10 @@
         <v>675</v>
       </c>
       <c r="B594" s="1">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="C594" s="1" t="s">
-        <v>24</v>
+        <v>229</v>
       </c>
       <c r="D594" s="3" t="s">
         <v>20</v>
@@ -10981,13 +10984,13 @@
     </row>
     <row r="595" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A595" s="1" t="s">
-        <v>316</v>
+        <v>675</v>
       </c>
       <c r="B595" s="1">
-        <v>75</v>
+        <v>50</v>
       </c>
       <c r="C595" s="1" t="s">
-        <v>492</v>
+        <v>24</v>
       </c>
       <c r="D595" s="3" t="s">
         <v>20</v>
@@ -10998,10 +11001,10 @@
         <v>316</v>
       </c>
       <c r="B596" s="1">
-        <v>55</v>
+        <v>75</v>
       </c>
       <c r="C596" s="1" t="s">
-        <v>236</v>
+        <v>492</v>
       </c>
       <c r="D596" s="3" t="s">
         <v>20</v>
@@ -11009,16 +11012,16 @@
     </row>
     <row r="597" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A597" s="1" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="B597" s="1">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="C597" s="1" t="s">
-        <v>23</v>
+        <v>236</v>
       </c>
       <c r="D597" s="3" t="s">
-        <v>26</v>
+        <v>20</v>
       </c>
     </row>
     <row r="598" spans="1:4" x14ac:dyDescent="0.45">
@@ -11029,10 +11032,10 @@
         <v>50</v>
       </c>
       <c r="C598" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D598" s="3" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="599" spans="1:4" x14ac:dyDescent="0.45">
@@ -11040,13 +11043,13 @@
         <v>317</v>
       </c>
       <c r="B599" s="1">
-        <v>1500</v>
+        <v>50</v>
       </c>
       <c r="C599" s="1" t="s">
-        <v>318</v>
+        <v>24</v>
       </c>
       <c r="D599" s="3" t="s">
-        <v>20</v>
+        <v>27</v>
       </c>
     </row>
     <row r="600" spans="1:4" x14ac:dyDescent="0.45">
@@ -11054,13 +11057,13 @@
         <v>317</v>
       </c>
       <c r="B600" s="1">
-        <v>60</v>
+        <v>1500</v>
       </c>
       <c r="C600" s="1" t="s">
-        <v>414</v>
+        <v>318</v>
       </c>
       <c r="D600" s="3" t="s">
-        <v>48</v>
+        <v>20</v>
       </c>
     </row>
     <row r="601" spans="1:4" x14ac:dyDescent="0.45">
@@ -11068,27 +11071,27 @@
         <v>317</v>
       </c>
       <c r="B601" s="1">
-        <v>20</v>
+        <v>60</v>
       </c>
       <c r="C601" s="1" t="s">
-        <v>464</v>
+        <v>414</v>
       </c>
       <c r="D601" s="3" t="s">
-        <v>22</v>
+        <v>48</v>
       </c>
     </row>
     <row r="602" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A602" s="1" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
       <c r="B602" s="1">
-        <v>100</v>
+        <v>20</v>
       </c>
       <c r="C602" s="1" t="s">
-        <v>24</v>
+        <v>464</v>
       </c>
       <c r="D602" s="3" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
     </row>
     <row r="603" spans="1:4" x14ac:dyDescent="0.45">
@@ -11096,10 +11099,10 @@
         <v>319</v>
       </c>
       <c r="B603" s="1">
-        <v>60</v>
+        <v>100</v>
       </c>
       <c r="C603" s="1" t="s">
-        <v>240</v>
+        <v>24</v>
       </c>
       <c r="D603" s="3" t="s">
         <v>20</v>
@@ -11110,13 +11113,13 @@
         <v>319</v>
       </c>
       <c r="B604" s="1">
-        <v>75</v>
+        <v>60</v>
       </c>
       <c r="C604" s="1" t="s">
-        <v>492</v>
+        <v>240</v>
       </c>
       <c r="D604" s="3" t="s">
-        <v>388</v>
+        <v>20</v>
       </c>
     </row>
     <row r="605" spans="1:4" x14ac:dyDescent="0.45">
@@ -11124,10 +11127,10 @@
         <v>319</v>
       </c>
       <c r="B605" s="1">
-        <v>225</v>
+        <v>75</v>
       </c>
       <c r="C605" s="1" t="s">
-        <v>493</v>
+        <v>492</v>
       </c>
       <c r="D605" s="3" t="s">
         <v>388</v>
@@ -11135,16 +11138,16 @@
     </row>
     <row r="606" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A606" s="1" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="B606" s="1">
-        <v>75</v>
+        <v>225</v>
       </c>
       <c r="C606" s="1" t="s">
         <v>493</v>
       </c>
       <c r="D606" s="3" t="s">
-        <v>20</v>
+        <v>388</v>
       </c>
     </row>
     <row r="607" spans="1:4" x14ac:dyDescent="0.45">
@@ -11152,13 +11155,13 @@
         <v>320</v>
       </c>
       <c r="B607" s="1">
-        <v>40</v>
+        <v>75</v>
       </c>
       <c r="C607" s="1" t="s">
-        <v>411</v>
+        <v>493</v>
       </c>
       <c r="D607" s="3" t="s">
-        <v>36</v>
+        <v>20</v>
       </c>
     </row>
     <row r="608" spans="1:4" x14ac:dyDescent="0.45">
@@ -11166,27 +11169,27 @@
         <v>320</v>
       </c>
       <c r="B608" s="1">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="C608" s="1" t="s">
-        <v>240</v>
+        <v>411</v>
       </c>
       <c r="D608" s="3" t="s">
-        <v>20</v>
+        <v>36</v>
       </c>
     </row>
     <row r="609" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A609" s="1" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="B609" s="1">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="C609" s="1" t="s">
-        <v>414</v>
+        <v>240</v>
       </c>
       <c r="D609" s="3" t="s">
-        <v>48</v>
+        <v>20</v>
       </c>
     </row>
     <row r="610" spans="1:5" x14ac:dyDescent="0.45">
@@ -11194,16 +11197,13 @@
         <v>321</v>
       </c>
       <c r="B610" s="1">
-        <v>54</v>
+        <v>20</v>
       </c>
       <c r="C610" s="1" t="s">
-        <v>240</v>
+        <v>414</v>
       </c>
       <c r="D610" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="E610" s="1" t="s">
-        <v>322</v>
+        <v>48</v>
       </c>
     </row>
     <row r="611" spans="1:5" x14ac:dyDescent="0.45">
@@ -11211,13 +11211,16 @@
         <v>321</v>
       </c>
       <c r="B611" s="1">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="C611" s="1" t="s">
-        <v>172</v>
+        <v>240</v>
       </c>
       <c r="D611" s="3" t="s">
         <v>20</v>
+      </c>
+      <c r="E611" s="1" t="s">
+        <v>322</v>
       </c>
     </row>
     <row r="612" spans="1:5" x14ac:dyDescent="0.45">
@@ -11225,13 +11228,13 @@
         <v>321</v>
       </c>
       <c r="B612" s="1">
-        <v>25</v>
+        <v>50</v>
       </c>
       <c r="C612" s="1" t="s">
-        <v>495</v>
+        <v>172</v>
       </c>
       <c r="D612" s="3" t="s">
-        <v>388</v>
+        <v>20</v>
       </c>
     </row>
     <row r="613" spans="1:5" x14ac:dyDescent="0.45">
@@ -11239,24 +11242,24 @@
         <v>321</v>
       </c>
       <c r="B613" s="1">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="C613" s="1" t="s">
-        <v>23</v>
+        <v>495</v>
       </c>
       <c r="D613" s="3" t="s">
-        <v>20</v>
+        <v>388</v>
       </c>
     </row>
     <row r="614" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A614" s="1" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
       <c r="B614" s="1">
-        <v>25</v>
+        <v>50</v>
       </c>
       <c r="C614" s="1" t="s">
-        <v>496</v>
+        <v>23</v>
       </c>
       <c r="D614" s="3" t="s">
         <v>20</v>
@@ -11267,10 +11270,10 @@
         <v>323</v>
       </c>
       <c r="B615" s="1">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="C615" s="1" t="s">
-        <v>493</v>
+        <v>496</v>
       </c>
       <c r="D615" s="3" t="s">
         <v>20</v>
@@ -11281,10 +11284,10 @@
         <v>323</v>
       </c>
       <c r="B616" s="1">
-        <v>620</v>
+        <v>50</v>
       </c>
       <c r="C616" s="1" t="s">
-        <v>324</v>
+        <v>493</v>
       </c>
       <c r="D616" s="3" t="s">
         <v>20</v>
@@ -11295,10 +11298,10 @@
         <v>323</v>
       </c>
       <c r="B617" s="1">
-        <v>100</v>
+        <v>620</v>
       </c>
       <c r="C617" s="1" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="D617" s="3" t="s">
         <v>20</v>
@@ -11309,10 +11312,10 @@
         <v>323</v>
       </c>
       <c r="B618" s="1">
-        <v>30</v>
+        <v>100</v>
       </c>
       <c r="C618" s="1" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="D618" s="3" t="s">
         <v>20</v>
@@ -11320,16 +11323,16 @@
     </row>
     <row r="619" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A619" s="1" t="s">
-        <v>327</v>
+        <v>323</v>
       </c>
       <c r="B619" s="1">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="C619" s="1" t="s">
-        <v>414</v>
+        <v>326</v>
       </c>
       <c r="D619" s="3" t="s">
-        <v>48</v>
+        <v>20</v>
       </c>
     </row>
     <row r="620" spans="1:5" x14ac:dyDescent="0.45">
@@ -11337,13 +11340,13 @@
         <v>327</v>
       </c>
       <c r="B620" s="1">
-        <v>60</v>
+        <v>20</v>
       </c>
       <c r="C620" s="1" t="s">
-        <v>464</v>
+        <v>414</v>
       </c>
       <c r="D620" s="3" t="s">
-        <v>22</v>
+        <v>48</v>
       </c>
     </row>
     <row r="621" spans="1:5" x14ac:dyDescent="0.45">
@@ -11354,10 +11357,10 @@
         <v>60</v>
       </c>
       <c r="C621" s="1" t="s">
-        <v>328</v>
+        <v>464</v>
       </c>
       <c r="D621" s="3" t="s">
-        <v>35</v>
+        <v>22</v>
       </c>
     </row>
     <row r="622" spans="1:5" x14ac:dyDescent="0.45">
@@ -11365,13 +11368,13 @@
         <v>327</v>
       </c>
       <c r="B622" s="1">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="C622" s="1" t="s">
-        <v>24</v>
+        <v>328</v>
       </c>
       <c r="D622" s="3" t="s">
-        <v>27</v>
+        <v>35</v>
       </c>
     </row>
     <row r="623" spans="1:5" x14ac:dyDescent="0.45">
@@ -11379,27 +11382,27 @@
         <v>327</v>
       </c>
       <c r="B623" s="1">
-        <v>25</v>
+        <v>50</v>
       </c>
       <c r="C623" s="1" t="s">
-        <v>57</v>
+        <v>24</v>
       </c>
       <c r="D623" s="3" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="624" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A624" s="1" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="B624" s="1">
         <v>25</v>
       </c>
       <c r="C624" s="1" t="s">
-        <v>24</v>
+        <v>57</v>
       </c>
       <c r="D624" s="3" t="s">
-        <v>20</v>
+        <v>26</v>
       </c>
     </row>
     <row r="625" spans="1:4" x14ac:dyDescent="0.45">
@@ -11407,7 +11410,7 @@
         <v>329</v>
       </c>
       <c r="B625" s="1">
-        <v>225</v>
+        <v>25</v>
       </c>
       <c r="C625" s="1" t="s">
         <v>24</v>
@@ -11421,13 +11424,13 @@
         <v>329</v>
       </c>
       <c r="B626" s="1">
-        <v>325</v>
+        <v>225</v>
       </c>
       <c r="C626" s="1" t="s">
-        <v>493</v>
+        <v>24</v>
       </c>
       <c r="D626" s="3" t="s">
-        <v>388</v>
+        <v>20</v>
       </c>
     </row>
     <row r="627" spans="1:4" x14ac:dyDescent="0.45">
@@ -11435,13 +11438,13 @@
         <v>329</v>
       </c>
       <c r="B627" s="1">
-        <v>28</v>
+        <v>325</v>
       </c>
       <c r="C627" s="1" t="s">
-        <v>19</v>
+        <v>493</v>
       </c>
       <c r="D627" s="3" t="s">
-        <v>20</v>
+        <v>388</v>
       </c>
     </row>
     <row r="628" spans="1:4" x14ac:dyDescent="0.45">
@@ -11449,10 +11452,10 @@
         <v>329</v>
       </c>
       <c r="B628" s="1">
-        <v>180</v>
+        <v>28</v>
       </c>
       <c r="C628" s="1" t="s">
-        <v>229</v>
+        <v>19</v>
       </c>
       <c r="D628" s="3" t="s">
         <v>20</v>
@@ -11463,13 +11466,13 @@
         <v>329</v>
       </c>
       <c r="B629" s="1">
-        <v>140</v>
+        <v>180</v>
       </c>
       <c r="C629" s="1" t="s">
-        <v>414</v>
+        <v>229</v>
       </c>
       <c r="D629" s="3" t="s">
-        <v>48</v>
+        <v>20</v>
       </c>
     </row>
     <row r="630" spans="1:4" x14ac:dyDescent="0.45">
@@ -11477,13 +11480,13 @@
         <v>329</v>
       </c>
       <c r="B630" s="1">
-        <v>150</v>
+        <v>140</v>
       </c>
       <c r="C630" s="1" t="s">
-        <v>21</v>
+        <v>414</v>
       </c>
       <c r="D630" s="3" t="s">
-        <v>20</v>
+        <v>48</v>
       </c>
     </row>
     <row r="631" spans="1:4" x14ac:dyDescent="0.45">
@@ -11491,10 +11494,10 @@
         <v>329</v>
       </c>
       <c r="B631" s="1">
-        <v>50</v>
+        <v>150</v>
       </c>
       <c r="C631" s="1" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="D631" s="3" t="s">
         <v>20</v>
@@ -11505,13 +11508,13 @@
         <v>329</v>
       </c>
       <c r="B632" s="1">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="C632" s="1" t="s">
-        <v>89</v>
+        <v>23</v>
       </c>
       <c r="D632" s="3" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
     <row r="633" spans="1:4" x14ac:dyDescent="0.45">
@@ -11519,10 +11522,10 @@
         <v>329</v>
       </c>
       <c r="B633" s="1">
-        <v>120</v>
+        <v>100</v>
       </c>
       <c r="C633" s="1" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D633" s="3" t="s">
         <v>22</v>
@@ -11533,10 +11536,10 @@
         <v>329</v>
       </c>
       <c r="B634" s="1">
-        <v>620</v>
+        <v>120</v>
       </c>
       <c r="C634" s="1" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="D634" s="3" t="s">
         <v>22</v>
@@ -11547,10 +11550,10 @@
         <v>329</v>
       </c>
       <c r="B635" s="1">
-        <v>50</v>
+        <v>620</v>
       </c>
       <c r="C635" s="1" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="D635" s="3" t="s">
         <v>22</v>
@@ -11558,16 +11561,16 @@
     </row>
     <row r="636" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A636" s="1" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="B636" s="1">
         <v>50</v>
       </c>
       <c r="C636" s="1" t="s">
-        <v>497</v>
+        <v>91</v>
       </c>
       <c r="D636" s="3" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
     </row>
     <row r="637" spans="1:4" x14ac:dyDescent="0.45">
@@ -11575,10 +11578,10 @@
         <v>330</v>
       </c>
       <c r="B637" s="1">
-        <v>243</v>
+        <v>50</v>
       </c>
       <c r="C637" s="1" t="s">
-        <v>19</v>
+        <v>497</v>
       </c>
       <c r="D637" s="3" t="s">
         <v>20</v>
@@ -11589,10 +11592,10 @@
         <v>330</v>
       </c>
       <c r="B638" s="1">
-        <v>100</v>
+        <v>243</v>
       </c>
       <c r="C638" s="1" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="D638" s="3" t="s">
         <v>20</v>
@@ -11603,10 +11606,10 @@
         <v>330</v>
       </c>
       <c r="B639" s="1">
-        <v>30</v>
+        <v>100</v>
       </c>
       <c r="C639" s="1" t="s">
-        <v>33</v>
+        <v>24</v>
       </c>
       <c r="D639" s="3" t="s">
         <v>20</v>
@@ -11614,21 +11617,21 @@
     </row>
     <row r="640" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A640" s="1" t="s">
-        <v>331</v>
+        <v>330</v>
+      </c>
+      <c r="B640" s="1">
+        <v>30</v>
+      </c>
+      <c r="C640" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="D640" s="3" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="641" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A641" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="B641" s="1">
-        <v>90</v>
-      </c>
-      <c r="C641" s="1" t="s">
-        <v>87</v>
-      </c>
-      <c r="D641" s="3" t="s">
-        <v>35</v>
+        <v>331</v>
       </c>
     </row>
     <row r="642" spans="1:4" x14ac:dyDescent="0.45">
@@ -11636,13 +11639,13 @@
         <v>11</v>
       </c>
       <c r="B642" s="1">
-        <v>25</v>
+        <v>90</v>
       </c>
       <c r="C642" s="1" t="s">
-        <v>99</v>
+        <v>87</v>
       </c>
       <c r="D642" s="3" t="s">
-        <v>22</v>
+        <v>35</v>
       </c>
     </row>
     <row r="643" spans="1:4" x14ac:dyDescent="0.45">
@@ -11650,13 +11653,13 @@
         <v>11</v>
       </c>
       <c r="B643" s="1">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="C643" s="1" t="s">
-        <v>414</v>
+        <v>99</v>
       </c>
       <c r="D643" s="3" t="s">
-        <v>48</v>
+        <v>22</v>
       </c>
     </row>
     <row r="644" spans="1:4" x14ac:dyDescent="0.45">
@@ -11664,13 +11667,13 @@
         <v>11</v>
       </c>
       <c r="B644" s="1">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="C644" s="1" t="s">
-        <v>23</v>
+        <v>414</v>
       </c>
       <c r="D644" s="3" t="s">
-        <v>26</v>
+        <v>48</v>
       </c>
     </row>
     <row r="645" spans="1:4" x14ac:dyDescent="0.45">
@@ -11678,13 +11681,13 @@
         <v>11</v>
       </c>
       <c r="B645" s="1">
-        <v>25</v>
+        <v>50</v>
       </c>
       <c r="C645" s="1" t="s">
-        <v>257</v>
+        <v>23</v>
       </c>
       <c r="D645" s="3" t="s">
-        <v>39</v>
+        <v>26</v>
       </c>
     </row>
     <row r="646" spans="1:4" x14ac:dyDescent="0.45">
@@ -11695,10 +11698,10 @@
         <v>25</v>
       </c>
       <c r="C646" s="1" t="s">
-        <v>332</v>
+        <v>257</v>
       </c>
       <c r="D646" s="3" t="s">
-        <v>390</v>
+        <v>39</v>
       </c>
     </row>
     <row r="647" spans="1:4" x14ac:dyDescent="0.45">
@@ -11706,41 +11709,41 @@
         <v>11</v>
       </c>
       <c r="B647" s="1">
-        <v>100</v>
+        <v>25</v>
       </c>
       <c r="C647" s="1" t="s">
-        <v>498</v>
+        <v>332</v>
       </c>
       <c r="D647" s="3" t="s">
-        <v>22</v>
+        <v>390</v>
       </c>
     </row>
     <row r="648" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A648" s="1" t="s">
-        <v>333</v>
+        <v>11</v>
       </c>
       <c r="B648" s="1">
         <v>100</v>
       </c>
       <c r="C648" s="1" t="s">
-        <v>493</v>
+        <v>498</v>
       </c>
       <c r="D648" s="3" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
     </row>
     <row r="649" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A649" s="1" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="B649" s="1">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="C649" s="1" t="s">
-        <v>391</v>
+        <v>493</v>
       </c>
       <c r="D649" s="3" t="s">
-        <v>35</v>
+        <v>20</v>
       </c>
     </row>
     <row r="650" spans="1:4" x14ac:dyDescent="0.45">
@@ -11748,13 +11751,13 @@
         <v>334</v>
       </c>
       <c r="B650" s="1">
-        <v>20</v>
+        <v>50</v>
       </c>
       <c r="C650" s="1" t="s">
-        <v>499</v>
+        <v>391</v>
       </c>
       <c r="D650" s="3" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="651" spans="1:4" x14ac:dyDescent="0.45">
@@ -11762,27 +11765,27 @@
         <v>334</v>
       </c>
       <c r="B651" s="1">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="C651" s="1" t="s">
-        <v>118</v>
+        <v>499</v>
       </c>
       <c r="D651" s="3" t="s">
-        <v>22</v>
+        <v>36</v>
       </c>
     </row>
     <row r="652" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A652" s="1" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="B652" s="1">
         <v>50</v>
       </c>
       <c r="C652" s="1" t="s">
-        <v>493</v>
+        <v>118</v>
       </c>
       <c r="D652" s="3" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
     </row>
     <row r="653" spans="1:4" x14ac:dyDescent="0.45">
@@ -11790,10 +11793,10 @@
         <v>335</v>
       </c>
       <c r="B653" s="1">
-        <v>155</v>
+        <v>50</v>
       </c>
       <c r="C653" s="1" t="s">
-        <v>19</v>
+        <v>493</v>
       </c>
       <c r="D653" s="3" t="s">
         <v>20</v>
@@ -11804,27 +11807,27 @@
         <v>335</v>
       </c>
       <c r="B654" s="1">
-        <v>25</v>
+        <v>155</v>
       </c>
       <c r="C654" s="1" t="s">
-        <v>99</v>
+        <v>19</v>
       </c>
       <c r="D654" s="3" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
     <row r="655" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A655" s="1" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="B655" s="1">
-        <v>75</v>
+        <v>25</v>
       </c>
       <c r="C655" s="1" t="s">
-        <v>337</v>
+        <v>99</v>
       </c>
       <c r="D655" s="3" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
     </row>
     <row r="656" spans="1:4" x14ac:dyDescent="0.45">
@@ -11835,7 +11838,7 @@
         <v>75</v>
       </c>
       <c r="C656" s="1" t="s">
-        <v>500</v>
+        <v>337</v>
       </c>
       <c r="D656" s="3" t="s">
         <v>20</v>
@@ -11846,10 +11849,10 @@
         <v>336</v>
       </c>
       <c r="B657" s="1">
-        <v>50</v>
+        <v>75</v>
       </c>
       <c r="C657" s="1" t="s">
-        <v>501</v>
+        <v>500</v>
       </c>
       <c r="D657" s="3" t="s">
         <v>20</v>
@@ -11860,27 +11863,27 @@
         <v>336</v>
       </c>
       <c r="B658" s="1">
-        <v>500</v>
+        <v>50</v>
       </c>
       <c r="C658" s="1" t="s">
-        <v>38</v>
+        <v>501</v>
       </c>
       <c r="D658" s="3" t="s">
-        <v>39</v>
+        <v>20</v>
       </c>
     </row>
     <row r="659" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A659" s="1" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="B659" s="1">
-        <v>40</v>
+        <v>500</v>
       </c>
       <c r="C659" s="1" t="s">
-        <v>415</v>
+        <v>38</v>
       </c>
       <c r="D659" s="3" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
     </row>
     <row r="660" spans="1:4" x14ac:dyDescent="0.45">
@@ -11888,41 +11891,41 @@
         <v>338</v>
       </c>
       <c r="B660" s="1">
-        <v>75</v>
+        <v>40</v>
       </c>
       <c r="C660" s="1" t="s">
-        <v>23</v>
+        <v>415</v>
       </c>
       <c r="D660" s="3" t="s">
-        <v>26</v>
+        <v>36</v>
       </c>
     </row>
     <row r="661" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A661" s="1" t="s">
-        <v>8</v>
+        <v>338</v>
       </c>
       <c r="B661" s="1">
-        <v>447</v>
+        <v>75</v>
       </c>
       <c r="C661" s="1" t="s">
-        <v>339</v>
+        <v>23</v>
       </c>
       <c r="D661" s="3" t="s">
-        <v>20</v>
+        <v>26</v>
       </c>
     </row>
     <row r="662" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A662" s="1" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="B662" s="1">
-        <v>25</v>
+        <v>447</v>
       </c>
       <c r="C662" s="1" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="D662" s="3" t="s">
-        <v>26</v>
+        <v>20</v>
       </c>
     </row>
     <row r="663" spans="1:4" x14ac:dyDescent="0.45">
@@ -11930,13 +11933,13 @@
         <v>12</v>
       </c>
       <c r="B663" s="1">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="C663" s="1" t="s">
-        <v>502</v>
+        <v>340</v>
       </c>
       <c r="D663" s="3" t="s">
-        <v>388</v>
+        <v>26</v>
       </c>
     </row>
     <row r="664" spans="1:4" x14ac:dyDescent="0.45">
@@ -11944,13 +11947,13 @@
         <v>12</v>
       </c>
       <c r="B664" s="1">
-        <v>20</v>
+        <v>50</v>
       </c>
       <c r="C664" s="1" t="s">
-        <v>464</v>
+        <v>502</v>
       </c>
       <c r="D664" s="3" t="s">
-        <v>22</v>
+        <v>388</v>
       </c>
     </row>
     <row r="665" spans="1:4" x14ac:dyDescent="0.45">
@@ -11958,13 +11961,13 @@
         <v>12</v>
       </c>
       <c r="B665" s="1">
-        <v>100</v>
+        <v>20</v>
       </c>
       <c r="C665" s="1" t="s">
-        <v>21</v>
+        <v>464</v>
       </c>
       <c r="D665" s="3" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
     </row>
     <row r="666" spans="1:4" x14ac:dyDescent="0.45">
@@ -11972,13 +11975,13 @@
         <v>12</v>
       </c>
       <c r="B666" s="1">
-        <v>150</v>
+        <v>100</v>
       </c>
       <c r="C666" s="1" t="s">
-        <v>341</v>
+        <v>21</v>
       </c>
       <c r="D666" s="3" t="s">
-        <v>292</v>
+        <v>25</v>
       </c>
     </row>
     <row r="667" spans="1:4" x14ac:dyDescent="0.45">
@@ -11986,13 +11989,13 @@
         <v>12</v>
       </c>
       <c r="B667" s="1">
-        <v>50</v>
+        <v>150</v>
       </c>
       <c r="C667" s="1" t="s">
-        <v>337</v>
+        <v>341</v>
       </c>
       <c r="D667" s="3" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
     </row>
     <row r="668" spans="1:4" x14ac:dyDescent="0.45">
@@ -12000,27 +12003,27 @@
         <v>12</v>
       </c>
       <c r="B668" s="1">
-        <v>25</v>
+        <v>50</v>
       </c>
       <c r="C668" s="1" t="s">
-        <v>342</v>
+        <v>337</v>
       </c>
       <c r="D668" s="3" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
     </row>
     <row r="669" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A669" s="1" t="s">
-        <v>343</v>
+        <v>12</v>
       </c>
       <c r="B669" s="1">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="C669" s="1" t="s">
-        <v>492</v>
+        <v>342</v>
       </c>
       <c r="D669" s="3" t="s">
-        <v>20</v>
+        <v>288</v>
       </c>
     </row>
     <row r="670" spans="1:4" x14ac:dyDescent="0.45">
@@ -12028,10 +12031,10 @@
         <v>343</v>
       </c>
       <c r="B670" s="1">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="C670" s="1" t="s">
-        <v>21</v>
+        <v>492</v>
       </c>
       <c r="D670" s="3" t="s">
         <v>20</v>
@@ -12039,13 +12042,13 @@
     </row>
     <row r="671" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A671" s="1" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="B671" s="1">
-        <v>75</v>
+        <v>100</v>
       </c>
       <c r="C671" s="1" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="D671" s="3" t="s">
         <v>20</v>
@@ -12056,13 +12059,13 @@
         <v>344</v>
       </c>
       <c r="B672" s="1">
-        <v>40</v>
+        <v>75</v>
       </c>
       <c r="C672" s="1" t="s">
-        <v>491</v>
+        <v>24</v>
       </c>
       <c r="D672" s="3" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
     <row r="673" spans="1:4" x14ac:dyDescent="0.45">
@@ -12070,10 +12073,10 @@
         <v>344</v>
       </c>
       <c r="B673" s="1">
-        <v>25</v>
+        <v>40</v>
       </c>
       <c r="C673" s="1" t="s">
-        <v>99</v>
+        <v>491</v>
       </c>
       <c r="D673" s="3" t="s">
         <v>22</v>
@@ -12084,13 +12087,13 @@
         <v>344</v>
       </c>
       <c r="B674" s="1">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="C674" s="1" t="s">
-        <v>414</v>
+        <v>99</v>
       </c>
       <c r="D674" s="3" t="s">
-        <v>48</v>
+        <v>22</v>
       </c>
     </row>
     <row r="675" spans="1:4" x14ac:dyDescent="0.45">
@@ -12101,24 +12104,24 @@
         <v>20</v>
       </c>
       <c r="C675" s="1" t="s">
-        <v>411</v>
+        <v>414</v>
       </c>
       <c r="D675" s="3" t="s">
-        <v>36</v>
+        <v>48</v>
       </c>
     </row>
     <row r="676" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A676" s="1" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="B676" s="1">
-        <v>150</v>
+        <v>20</v>
       </c>
       <c r="C676" s="1" t="s">
-        <v>503</v>
+        <v>411</v>
       </c>
       <c r="D676" s="3" t="s">
-        <v>388</v>
+        <v>36</v>
       </c>
     </row>
     <row r="677" spans="1:4" x14ac:dyDescent="0.45">
@@ -12126,13 +12129,13 @@
         <v>345</v>
       </c>
       <c r="B677" s="1">
-        <v>25</v>
+        <v>150</v>
       </c>
       <c r="C677" s="1" t="s">
-        <v>504</v>
+        <v>503</v>
       </c>
       <c r="D677" s="3" t="s">
-        <v>392</v>
+        <v>388</v>
       </c>
     </row>
     <row r="678" spans="1:4" x14ac:dyDescent="0.45">
@@ -12143,24 +12146,24 @@
         <v>25</v>
       </c>
       <c r="C678" s="1" t="s">
-        <v>505</v>
+        <v>504</v>
       </c>
       <c r="D678" s="3" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
     </row>
     <row r="679" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A679" s="1" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="B679" s="1">
-        <v>40</v>
+        <v>25</v>
       </c>
       <c r="C679" s="1" t="s">
-        <v>414</v>
+        <v>505</v>
       </c>
       <c r="D679" s="3" t="s">
-        <v>48</v>
+        <v>393</v>
       </c>
     </row>
     <row r="680" spans="1:4" x14ac:dyDescent="0.45">
@@ -12168,13 +12171,13 @@
         <v>346</v>
       </c>
       <c r="B680" s="1">
-        <v>201</v>
+        <v>40</v>
       </c>
       <c r="C680" s="1" t="s">
-        <v>19</v>
+        <v>414</v>
       </c>
       <c r="D680" s="3" t="s">
-        <v>20</v>
+        <v>48</v>
       </c>
     </row>
     <row r="681" spans="1:4" x14ac:dyDescent="0.45">
@@ -12182,13 +12185,13 @@
         <v>346</v>
       </c>
       <c r="B681" s="1">
-        <v>50</v>
+        <v>201</v>
       </c>
       <c r="C681" s="1" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="D681" s="3" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
     </row>
     <row r="682" spans="1:4" x14ac:dyDescent="0.45">
@@ -12196,13 +12199,13 @@
         <v>346</v>
       </c>
       <c r="B682" s="1">
-        <v>1100</v>
+        <v>50</v>
       </c>
       <c r="C682" s="1" t="s">
-        <v>646</v>
+        <v>24</v>
       </c>
       <c r="D682" s="3" t="s">
-        <v>20</v>
+        <v>27</v>
       </c>
     </row>
     <row r="683" spans="1:4" x14ac:dyDescent="0.45">
@@ -12210,10 +12213,10 @@
         <v>346</v>
       </c>
       <c r="B683" s="1">
-        <v>900</v>
+        <v>1100</v>
       </c>
       <c r="C683" s="1" t="s">
-        <v>647</v>
+        <v>646</v>
       </c>
       <c r="D683" s="3" t="s">
         <v>20</v>
@@ -12224,13 +12227,13 @@
         <v>346</v>
       </c>
       <c r="B684" s="1">
-        <v>20</v>
+        <v>900</v>
       </c>
       <c r="C684" s="1" t="s">
-        <v>411</v>
+        <v>647</v>
       </c>
       <c r="D684" s="3" t="s">
-        <v>36</v>
+        <v>20</v>
       </c>
     </row>
     <row r="685" spans="1:4" x14ac:dyDescent="0.45">
@@ -12241,10 +12244,10 @@
         <v>20</v>
       </c>
       <c r="C685" s="1" t="s">
-        <v>506</v>
+        <v>411</v>
       </c>
       <c r="D685" s="3" t="s">
-        <v>394</v>
+        <v>36</v>
       </c>
     </row>
     <row r="686" spans="1:4" x14ac:dyDescent="0.45">
@@ -12252,10 +12255,10 @@
         <v>346</v>
       </c>
       <c r="B686" s="1">
-        <v>291</v>
+        <v>20</v>
       </c>
       <c r="C686" s="1" t="s">
-        <v>347</v>
+        <v>506</v>
       </c>
       <c r="D686" s="3" t="s">
         <v>394</v>
@@ -12263,21 +12266,21 @@
     </row>
     <row r="687" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A687" s="1" t="s">
-        <v>348</v>
+        <v>346</v>
+      </c>
+      <c r="B687" s="1">
+        <v>291</v>
+      </c>
+      <c r="C687" s="1" t="s">
+        <v>347</v>
+      </c>
+      <c r="D687" s="3" t="s">
+        <v>394</v>
       </c>
     </row>
     <row r="688" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A688" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B688" s="1">
-        <v>250</v>
-      </c>
-      <c r="C688" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="D688" s="3" t="s">
-        <v>25</v>
+        <v>348</v>
       </c>
     </row>
     <row r="689" spans="1:4" x14ac:dyDescent="0.45">
@@ -12285,13 +12288,13 @@
         <v>9</v>
       </c>
       <c r="B689" s="1">
-        <v>275</v>
+        <v>250</v>
       </c>
       <c r="C689" s="1" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="D689" s="3" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
     </row>
     <row r="690" spans="1:4" x14ac:dyDescent="0.45">
@@ -12299,13 +12302,13 @@
         <v>9</v>
       </c>
       <c r="B690" s="1">
-        <v>115</v>
+        <v>275</v>
       </c>
       <c r="C690" s="1" t="s">
-        <v>33</v>
+        <v>24</v>
       </c>
       <c r="D690" s="3" t="s">
-        <v>35</v>
+        <v>27</v>
       </c>
     </row>
     <row r="691" spans="1:4" x14ac:dyDescent="0.45">
@@ -12313,13 +12316,13 @@
         <v>9</v>
       </c>
       <c r="B691" s="1">
-        <v>75</v>
+        <v>115</v>
       </c>
       <c r="C691" s="1" t="s">
-        <v>418</v>
+        <v>33</v>
       </c>
       <c r="D691" s="3" t="s">
-        <v>48</v>
+        <v>35</v>
       </c>
     </row>
     <row r="692" spans="1:4" x14ac:dyDescent="0.45">
@@ -12327,13 +12330,13 @@
         <v>9</v>
       </c>
       <c r="B692" s="1">
-        <v>60</v>
+        <v>75</v>
       </c>
       <c r="C692" s="1" t="s">
-        <v>507</v>
+        <v>418</v>
       </c>
       <c r="D692" s="3" t="s">
-        <v>402</v>
+        <v>48</v>
       </c>
     </row>
     <row r="693" spans="1:4" x14ac:dyDescent="0.45">
@@ -12341,13 +12344,13 @@
         <v>9</v>
       </c>
       <c r="B693" s="1">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="C693" s="1" t="s">
-        <v>508</v>
+        <v>507</v>
       </c>
       <c r="D693" s="3" t="s">
-        <v>395</v>
+        <v>402</v>
       </c>
     </row>
     <row r="694" spans="1:4" x14ac:dyDescent="0.45">
@@ -12355,13 +12358,13 @@
         <v>9</v>
       </c>
       <c r="B694" s="1">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="C694" s="1" t="s">
-        <v>23</v>
+        <v>508</v>
       </c>
       <c r="D694" s="3" t="s">
-        <v>26</v>
+        <v>395</v>
       </c>
     </row>
     <row r="695" spans="1:4" x14ac:dyDescent="0.45">
@@ -12369,13 +12372,13 @@
         <v>9</v>
       </c>
       <c r="B695" s="1">
-        <v>25</v>
+        <v>100</v>
       </c>
       <c r="C695" s="1" t="s">
-        <v>99</v>
+        <v>23</v>
       </c>
       <c r="D695" s="3" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
     </row>
     <row r="696" spans="1:4" x14ac:dyDescent="0.45">
@@ -12383,10 +12386,10 @@
         <v>9</v>
       </c>
       <c r="B696" s="1">
-        <v>75</v>
+        <v>25</v>
       </c>
       <c r="C696" s="1" t="s">
-        <v>349</v>
+        <v>99</v>
       </c>
       <c r="D696" s="3" t="s">
         <v>22</v>
@@ -12397,24 +12400,24 @@
         <v>9</v>
       </c>
       <c r="B697" s="1">
-        <v>100</v>
+        <v>75</v>
       </c>
       <c r="C697" s="1" t="s">
-        <v>488</v>
+        <v>349</v>
       </c>
       <c r="D697" s="3" t="s">
-        <v>395</v>
+        <v>22</v>
       </c>
     </row>
     <row r="698" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A698" s="1" t="s">
-        <v>676</v>
+        <v>9</v>
       </c>
       <c r="B698" s="1">
-        <v>20</v>
+        <v>100</v>
       </c>
       <c r="C698" s="1" t="s">
-        <v>509</v>
+        <v>488</v>
       </c>
       <c r="D698" s="3" t="s">
         <v>395</v>
@@ -12425,27 +12428,27 @@
         <v>676</v>
       </c>
       <c r="B699" s="1">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="C699" s="1" t="s">
-        <v>23</v>
+        <v>509</v>
       </c>
       <c r="D699" s="3" t="s">
-        <v>26</v>
+        <v>395</v>
       </c>
     </row>
     <row r="700" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A700" s="1" t="s">
-        <v>677</v>
+        <v>676</v>
       </c>
       <c r="B700" s="1">
-        <v>100</v>
+        <v>25</v>
       </c>
       <c r="C700" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D700" s="3" t="s">
-        <v>20</v>
+        <v>26</v>
       </c>
     </row>
     <row r="701" spans="1:4" x14ac:dyDescent="0.45">
@@ -12453,10 +12456,10 @@
         <v>677</v>
       </c>
       <c r="B701" s="1">
-        <v>75</v>
+        <v>100</v>
       </c>
       <c r="C701" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D701" s="3" t="s">
         <v>20</v>
@@ -12467,10 +12470,10 @@
         <v>677</v>
       </c>
       <c r="B702" s="1">
-        <v>40</v>
+        <v>75</v>
       </c>
       <c r="C702" s="1" t="s">
-        <v>509</v>
+        <v>23</v>
       </c>
       <c r="D702" s="3" t="s">
         <v>20</v>
@@ -12481,13 +12484,13 @@
         <v>677</v>
       </c>
       <c r="B703" s="1">
-        <v>150</v>
+        <v>40</v>
       </c>
       <c r="C703" s="1" t="s">
-        <v>21</v>
+        <v>509</v>
       </c>
       <c r="D703" s="3" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
     </row>
     <row r="704" spans="1:4" x14ac:dyDescent="0.45">
@@ -12495,13 +12498,13 @@
         <v>677</v>
       </c>
       <c r="B704" s="1">
-        <v>125</v>
+        <v>150</v>
       </c>
       <c r="C704" s="1" t="s">
-        <v>418</v>
+        <v>21</v>
       </c>
       <c r="D704" s="3" t="s">
-        <v>20</v>
+        <v>25</v>
       </c>
     </row>
     <row r="705" spans="1:5" x14ac:dyDescent="0.45">
@@ -12509,13 +12512,13 @@
         <v>677</v>
       </c>
       <c r="B705" s="1">
-        <v>60</v>
+        <v>125</v>
       </c>
       <c r="C705" s="1" t="s">
-        <v>33</v>
+        <v>418</v>
       </c>
       <c r="D705" s="3" t="s">
-        <v>35</v>
+        <v>20</v>
       </c>
     </row>
     <row r="706" spans="1:5" x14ac:dyDescent="0.45">
@@ -12523,13 +12526,13 @@
         <v>677</v>
       </c>
       <c r="B706" s="1">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="C706" s="1" t="s">
-        <v>488</v>
+        <v>33</v>
       </c>
       <c r="D706" s="3" t="s">
-        <v>20</v>
+        <v>35</v>
       </c>
     </row>
     <row r="707" spans="1:5" x14ac:dyDescent="0.45">
@@ -12537,30 +12540,27 @@
         <v>677</v>
       </c>
       <c r="B707" s="1">
-        <v>350</v>
+        <v>50</v>
       </c>
       <c r="C707" s="1" t="s">
-        <v>350</v>
+        <v>488</v>
       </c>
       <c r="D707" s="3" t="s">
-        <v>387</v>
+        <v>20</v>
       </c>
     </row>
     <row r="708" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A708" s="1" t="s">
-        <v>351</v>
+        <v>677</v>
       </c>
       <c r="B708" s="1">
-        <v>200</v>
+        <v>350</v>
       </c>
       <c r="C708" s="1" t="s">
-        <v>21</v>
+        <v>350</v>
       </c>
       <c r="D708" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="E708" s="1" t="s">
-        <v>353</v>
+        <v>387</v>
       </c>
     </row>
     <row r="709" spans="1:5" x14ac:dyDescent="0.45">
@@ -12568,13 +12568,16 @@
         <v>351</v>
       </c>
       <c r="B709" s="1">
-        <v>225</v>
+        <v>200</v>
       </c>
       <c r="C709" s="1" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="D709" s="3" t="s">
         <v>20</v>
+      </c>
+      <c r="E709" s="1" t="s">
+        <v>353</v>
       </c>
     </row>
     <row r="710" spans="1:5" x14ac:dyDescent="0.45">
@@ -12582,13 +12585,13 @@
         <v>351</v>
       </c>
       <c r="B710" s="1">
-        <v>1500</v>
+        <v>225</v>
       </c>
       <c r="C710" s="1" t="s">
-        <v>304</v>
+        <v>24</v>
       </c>
       <c r="D710" s="3" t="s">
-        <v>39</v>
+        <v>20</v>
       </c>
     </row>
     <row r="711" spans="1:5" x14ac:dyDescent="0.45">
@@ -12596,13 +12599,13 @@
         <v>351</v>
       </c>
       <c r="B711" s="1">
-        <v>30</v>
+        <v>1500</v>
       </c>
       <c r="C711" s="1" t="s">
-        <v>33</v>
+        <v>304</v>
       </c>
       <c r="D711" s="3" t="s">
-        <v>20</v>
+        <v>39</v>
       </c>
     </row>
     <row r="712" spans="1:5" x14ac:dyDescent="0.45">
@@ -12610,13 +12613,13 @@
         <v>351</v>
       </c>
       <c r="B712" s="1">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="C712" s="1" t="s">
-        <v>509</v>
+        <v>33</v>
       </c>
       <c r="D712" s="3" t="s">
-        <v>396</v>
+        <v>20</v>
       </c>
     </row>
     <row r="713" spans="1:5" x14ac:dyDescent="0.45">
@@ -12627,10 +12630,10 @@
         <v>20</v>
       </c>
       <c r="C713" s="1" t="s">
-        <v>510</v>
+        <v>509</v>
       </c>
       <c r="D713" s="3" t="s">
-        <v>20</v>
+        <v>396</v>
       </c>
     </row>
     <row r="714" spans="1:5" x14ac:dyDescent="0.45">
@@ -12641,10 +12644,10 @@
         <v>20</v>
       </c>
       <c r="C714" s="1" t="s">
-        <v>511</v>
+        <v>510</v>
       </c>
       <c r="D714" s="3" t="s">
-        <v>397</v>
+        <v>20</v>
       </c>
     </row>
     <row r="715" spans="1:5" x14ac:dyDescent="0.45">
@@ -12652,13 +12655,13 @@
         <v>351</v>
       </c>
       <c r="B715" s="1">
-        <v>75</v>
+        <v>20</v>
       </c>
       <c r="C715" s="1" t="s">
-        <v>23</v>
+        <v>511</v>
       </c>
       <c r="D715" s="3" t="s">
-        <v>20</v>
+        <v>397</v>
       </c>
     </row>
     <row r="716" spans="1:5" x14ac:dyDescent="0.45">
@@ -12666,27 +12669,27 @@
         <v>351</v>
       </c>
       <c r="B716" s="1">
-        <v>50</v>
+        <v>75</v>
       </c>
       <c r="C716" s="1" t="s">
-        <v>352</v>
+        <v>23</v>
       </c>
       <c r="D716" s="3" t="s">
-        <v>398</v>
+        <v>20</v>
       </c>
     </row>
     <row r="717" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A717" s="1" t="s">
-        <v>354</v>
+        <v>351</v>
       </c>
       <c r="B717" s="1">
-        <v>75</v>
+        <v>50</v>
       </c>
       <c r="C717" s="1" t="s">
-        <v>512</v>
+        <v>352</v>
       </c>
       <c r="D717" s="3" t="s">
-        <v>20</v>
+        <v>398</v>
       </c>
     </row>
     <row r="718" spans="1:5" x14ac:dyDescent="0.45">
@@ -12697,7 +12700,7 @@
         <v>75</v>
       </c>
       <c r="C718" s="1" t="s">
-        <v>24</v>
+        <v>512</v>
       </c>
       <c r="D718" s="3" t="s">
         <v>20</v>
@@ -12708,10 +12711,10 @@
         <v>354</v>
       </c>
       <c r="B719" s="1">
-        <v>50</v>
+        <v>75</v>
       </c>
       <c r="C719" s="1" t="s">
-        <v>57</v>
+        <v>24</v>
       </c>
       <c r="D719" s="3" t="s">
         <v>20</v>
@@ -12722,10 +12725,10 @@
         <v>354</v>
       </c>
       <c r="B720" s="1">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="C720" s="1" t="s">
-        <v>21</v>
+        <v>57</v>
       </c>
       <c r="D720" s="3" t="s">
         <v>20</v>
@@ -12736,10 +12739,10 @@
         <v>354</v>
       </c>
       <c r="B721" s="1">
-        <v>60</v>
+        <v>100</v>
       </c>
       <c r="C721" s="1" t="s">
-        <v>33</v>
+        <v>21</v>
       </c>
       <c r="D721" s="3" t="s">
         <v>20</v>
@@ -12747,13 +12750,13 @@
     </row>
     <row r="722" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A722" s="1" t="s">
-        <v>667</v>
+        <v>354</v>
       </c>
       <c r="B722" s="1">
-        <v>200</v>
+        <v>60</v>
       </c>
       <c r="C722" s="1" t="s">
-        <v>24</v>
+        <v>33</v>
       </c>
       <c r="D722" s="3" t="s">
         <v>20</v>
@@ -12764,10 +12767,10 @@
         <v>667</v>
       </c>
       <c r="B723" s="1">
-        <v>100</v>
+        <v>200</v>
       </c>
       <c r="C723" s="1" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="D723" s="3" t="s">
         <v>20</v>
@@ -12781,7 +12784,7 @@
         <v>100</v>
       </c>
       <c r="C724" s="1" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="D724" s="3" t="s">
         <v>20</v>
@@ -12792,10 +12795,10 @@
         <v>667</v>
       </c>
       <c r="B725" s="1">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="C725" s="1" t="s">
-        <v>87</v>
+        <v>23</v>
       </c>
       <c r="D725" s="3" t="s">
         <v>20</v>
@@ -12806,10 +12809,10 @@
         <v>667</v>
       </c>
       <c r="B726" s="1">
-        <v>5240</v>
+        <v>90</v>
       </c>
       <c r="C726" s="1" t="s">
-        <v>654</v>
+        <v>87</v>
       </c>
       <c r="D726" s="3" t="s">
         <v>20</v>
@@ -12820,10 +12823,10 @@
         <v>667</v>
       </c>
       <c r="B727" s="1">
-        <v>6980</v>
+        <v>5240</v>
       </c>
       <c r="C727" s="1" t="s">
-        <v>655</v>
+        <v>654</v>
       </c>
       <c r="D727" s="3" t="s">
         <v>20</v>
@@ -12834,13 +12837,13 @@
         <v>667</v>
       </c>
       <c r="B728" s="1">
-        <v>40</v>
+        <v>6980</v>
       </c>
       <c r="C728" s="1" t="s">
-        <v>525</v>
+        <v>655</v>
       </c>
       <c r="D728" s="3" t="s">
-        <v>405</v>
+        <v>20</v>
       </c>
     </row>
     <row r="729" spans="1:4" x14ac:dyDescent="0.45">
@@ -12848,13 +12851,13 @@
         <v>667</v>
       </c>
       <c r="B729" s="1">
-        <v>175</v>
+        <v>40</v>
       </c>
       <c r="C729" s="1" t="s">
-        <v>488</v>
+        <v>525</v>
       </c>
       <c r="D729" s="3" t="s">
-        <v>395</v>
+        <v>405</v>
       </c>
     </row>
     <row r="730" spans="1:4" x14ac:dyDescent="0.45">
@@ -12862,10 +12865,10 @@
         <v>667</v>
       </c>
       <c r="B730" s="1">
-        <v>20</v>
+        <v>175</v>
       </c>
       <c r="C730" s="1" t="s">
-        <v>668</v>
+        <v>488</v>
       </c>
       <c r="D730" s="3" t="s">
         <v>395</v>
@@ -12873,24 +12876,24 @@
     </row>
     <row r="731" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A731" s="1" t="s">
-        <v>666</v>
+        <v>667</v>
       </c>
       <c r="B731" s="1">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="C731" s="1" t="s">
-        <v>24</v>
+        <v>668</v>
       </c>
       <c r="D731" s="3" t="s">
-        <v>20</v>
+        <v>395</v>
       </c>
     </row>
     <row r="732" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A732" s="1" t="s">
-        <v>355</v>
+        <v>666</v>
       </c>
       <c r="B732" s="1">
-        <v>75</v>
+        <v>50</v>
       </c>
       <c r="C732" s="1" t="s">
         <v>24</v>
@@ -12904,10 +12907,10 @@
         <v>355</v>
       </c>
       <c r="B733" s="1">
-        <v>30</v>
+        <v>75</v>
       </c>
       <c r="C733" s="1" t="s">
-        <v>33</v>
+        <v>24</v>
       </c>
       <c r="D733" s="3" t="s">
         <v>20</v>
@@ -12918,27 +12921,27 @@
         <v>355</v>
       </c>
       <c r="B734" s="1">
-        <v>1500</v>
+        <v>30</v>
       </c>
       <c r="C734" s="1" t="s">
-        <v>356</v>
+        <v>33</v>
       </c>
       <c r="D734" s="3" t="s">
-        <v>399</v>
+        <v>20</v>
       </c>
     </row>
     <row r="735" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A735" s="1" t="s">
-        <v>357</v>
+        <v>355</v>
       </c>
       <c r="B735" s="1">
-        <v>100</v>
+        <v>1500</v>
       </c>
       <c r="C735" s="1" t="s">
-        <v>358</v>
+        <v>356</v>
       </c>
       <c r="D735" s="3" t="s">
-        <v>20</v>
+        <v>399</v>
       </c>
     </row>
     <row r="736" spans="1:4" x14ac:dyDescent="0.45">
@@ -12946,13 +12949,13 @@
         <v>357</v>
       </c>
       <c r="B736" s="1">
-        <v>40</v>
+        <v>100</v>
       </c>
       <c r="C736" s="1" t="s">
-        <v>510</v>
+        <v>358</v>
       </c>
       <c r="D736" s="3" t="s">
-        <v>402</v>
+        <v>20</v>
       </c>
     </row>
     <row r="737" spans="1:4" x14ac:dyDescent="0.45">
@@ -12960,10 +12963,10 @@
         <v>357</v>
       </c>
       <c r="B737" s="1">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="C737" s="1" t="s">
-        <v>507</v>
+        <v>510</v>
       </c>
       <c r="D737" s="3" t="s">
         <v>402</v>
@@ -12974,13 +12977,13 @@
         <v>357</v>
       </c>
       <c r="B738" s="1">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="C738" s="1" t="s">
-        <v>514</v>
+        <v>507</v>
       </c>
       <c r="D738" s="3" t="s">
-        <v>395</v>
+        <v>402</v>
       </c>
     </row>
     <row r="739" spans="1:4" x14ac:dyDescent="0.45">
@@ -12988,13 +12991,13 @@
         <v>357</v>
       </c>
       <c r="B739" s="1">
-        <v>20</v>
+        <v>50</v>
       </c>
       <c r="C739" s="1" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="D739" s="3" t="s">
-        <v>405</v>
+        <v>395</v>
       </c>
     </row>
     <row r="740" spans="1:4" x14ac:dyDescent="0.45">
@@ -13002,13 +13005,13 @@
         <v>357</v>
       </c>
       <c r="B740" s="1">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="C740" s="1" t="s">
-        <v>523</v>
+        <v>513</v>
       </c>
       <c r="D740" s="3" t="s">
-        <v>395</v>
+        <v>405</v>
       </c>
     </row>
     <row r="741" spans="1:4" x14ac:dyDescent="0.45">
@@ -13016,13 +13019,13 @@
         <v>357</v>
       </c>
       <c r="B741" s="1">
-        <v>75</v>
+        <v>40</v>
       </c>
       <c r="C741" s="1" t="s">
-        <v>418</v>
+        <v>523</v>
       </c>
       <c r="D741" s="3" t="s">
-        <v>48</v>
+        <v>395</v>
       </c>
     </row>
     <row r="742" spans="1:4" x14ac:dyDescent="0.45">
@@ -13033,10 +13036,10 @@
         <v>75</v>
       </c>
       <c r="C742" s="1" t="s">
-        <v>488</v>
+        <v>418</v>
       </c>
       <c r="D742" s="3" t="s">
-        <v>395</v>
+        <v>48</v>
       </c>
     </row>
     <row r="743" spans="1:4" x14ac:dyDescent="0.45">
@@ -13044,27 +13047,27 @@
         <v>357</v>
       </c>
       <c r="B743" s="1">
-        <v>25</v>
+        <v>75</v>
       </c>
       <c r="C743" s="1" t="s">
-        <v>242</v>
+        <v>488</v>
       </c>
       <c r="D743" s="3" t="s">
-        <v>397</v>
+        <v>395</v>
       </c>
     </row>
     <row r="744" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A744" s="1" t="s">
-        <v>679</v>
+        <v>357</v>
       </c>
       <c r="B744" s="1">
-        <v>75</v>
+        <v>25</v>
       </c>
       <c r="C744" s="1" t="s">
-        <v>418</v>
+        <v>242</v>
       </c>
       <c r="D744" s="3" t="s">
-        <v>20</v>
+        <v>397</v>
       </c>
     </row>
     <row r="745" spans="1:4" x14ac:dyDescent="0.45">
@@ -13072,13 +13075,13 @@
         <v>679</v>
       </c>
       <c r="B745" s="1">
-        <v>20</v>
+        <v>75</v>
       </c>
       <c r="C745" s="1" t="s">
-        <v>513</v>
+        <v>418</v>
       </c>
       <c r="D745" s="3" t="s">
-        <v>405</v>
+        <v>20</v>
       </c>
     </row>
     <row r="746" spans="1:4" x14ac:dyDescent="0.45">
@@ -13089,10 +13092,10 @@
         <v>20</v>
       </c>
       <c r="C746" s="1" t="s">
-        <v>509</v>
+        <v>513</v>
       </c>
       <c r="D746" s="3" t="s">
-        <v>20</v>
+        <v>405</v>
       </c>
     </row>
     <row r="747" spans="1:4" x14ac:dyDescent="0.45">
@@ -13100,10 +13103,10 @@
         <v>679</v>
       </c>
       <c r="B747" s="1">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="C747" s="1" t="s">
-        <v>24</v>
+        <v>509</v>
       </c>
       <c r="D747" s="3" t="s">
         <v>20</v>
@@ -13114,10 +13117,10 @@
         <v>679</v>
       </c>
       <c r="B748" s="1">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="C748" s="1" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="D748" s="3" t="s">
         <v>20</v>
@@ -13128,10 +13131,10 @@
         <v>679</v>
       </c>
       <c r="B749" s="1">
-        <v>25</v>
+        <v>100</v>
       </c>
       <c r="C749" s="1" t="s">
-        <v>57</v>
+        <v>21</v>
       </c>
       <c r="D749" s="3" t="s">
         <v>20</v>
@@ -13139,13 +13142,13 @@
     </row>
     <row r="750" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A750" s="1" t="s">
-        <v>359</v>
+        <v>679</v>
       </c>
       <c r="B750" s="1">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="C750" s="1" t="s">
-        <v>515</v>
+        <v>57</v>
       </c>
       <c r="D750" s="3" t="s">
         <v>20</v>
@@ -13156,10 +13159,10 @@
         <v>359</v>
       </c>
       <c r="B751" s="1">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="C751" s="1" t="s">
-        <v>509</v>
+        <v>515</v>
       </c>
       <c r="D751" s="3" t="s">
         <v>20</v>
@@ -13170,10 +13173,10 @@
         <v>359</v>
       </c>
       <c r="B752" s="1">
-        <v>100</v>
+        <v>40</v>
       </c>
       <c r="C752" s="1" t="s">
-        <v>488</v>
+        <v>509</v>
       </c>
       <c r="D752" s="3" t="s">
         <v>20</v>
@@ -13184,10 +13187,10 @@
         <v>359</v>
       </c>
       <c r="B753" s="1">
-        <v>16</v>
+        <v>100</v>
       </c>
       <c r="C753" s="1" t="s">
-        <v>19</v>
+        <v>488</v>
       </c>
       <c r="D753" s="3" t="s">
         <v>20</v>
@@ -13195,21 +13198,21 @@
     </row>
     <row r="754" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A754" s="1" t="s">
-        <v>360</v>
+        <v>359</v>
+      </c>
+      <c r="B754" s="1">
+        <v>16</v>
+      </c>
+      <c r="C754" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D754" s="3" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="755" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A755" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B755" s="1">
-        <v>225</v>
-      </c>
-      <c r="C755" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="D755" s="3" t="s">
-        <v>20</v>
+        <v>360</v>
       </c>
     </row>
     <row r="756" spans="1:4" x14ac:dyDescent="0.45">
@@ -13217,10 +13220,10 @@
         <v>10</v>
       </c>
       <c r="B756" s="1">
-        <v>475</v>
+        <v>225</v>
       </c>
       <c r="C756" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D756" s="3" t="s">
         <v>20</v>
@@ -13231,10 +13234,10 @@
         <v>10</v>
       </c>
       <c r="B757" s="1">
-        <v>150</v>
+        <v>475</v>
       </c>
       <c r="C757" s="1" t="s">
-        <v>87</v>
+        <v>24</v>
       </c>
       <c r="D757" s="3" t="s">
         <v>20</v>
@@ -13245,10 +13248,10 @@
         <v>10</v>
       </c>
       <c r="B758" s="1">
-        <v>18</v>
+        <v>150</v>
       </c>
       <c r="C758" s="1" t="s">
-        <v>19</v>
+        <v>87</v>
       </c>
       <c r="D758" s="3" t="s">
         <v>20</v>
@@ -13259,10 +13262,10 @@
         <v>10</v>
       </c>
       <c r="B759" s="1">
-        <v>40</v>
+        <v>18</v>
       </c>
       <c r="C759" s="1" t="s">
-        <v>510</v>
+        <v>19</v>
       </c>
       <c r="D759" s="3" t="s">
         <v>20</v>
@@ -13276,7 +13279,7 @@
         <v>40</v>
       </c>
       <c r="C760" s="1" t="s">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="D760" s="3" t="s">
         <v>20</v>
@@ -13287,13 +13290,13 @@
         <v>10</v>
       </c>
       <c r="B761" s="1">
-        <v>80</v>
+        <v>40</v>
       </c>
       <c r="C761" s="1" t="s">
-        <v>513</v>
+        <v>509</v>
       </c>
       <c r="D761" s="3" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
     <row r="762" spans="1:4" x14ac:dyDescent="0.45">
@@ -13301,10 +13304,10 @@
         <v>10</v>
       </c>
       <c r="B762" s="1">
-        <v>30</v>
+        <v>80</v>
       </c>
       <c r="C762" s="1" t="s">
-        <v>361</v>
+        <v>513</v>
       </c>
       <c r="D762" s="3" t="s">
         <v>22</v>
@@ -13315,10 +13318,10 @@
         <v>10</v>
       </c>
       <c r="B763" s="1">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="C763" s="1" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="D763" s="3" t="s">
         <v>22</v>
@@ -13326,16 +13329,16 @@
     </row>
     <row r="764" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A764" s="1" t="s">
-        <v>363</v>
+        <v>10</v>
       </c>
       <c r="B764" s="1">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="C764" s="1" t="s">
-        <v>516</v>
+        <v>362</v>
       </c>
       <c r="D764" s="3" t="s">
-        <v>405</v>
+        <v>22</v>
       </c>
     </row>
     <row r="765" spans="1:4" x14ac:dyDescent="0.45">
@@ -13343,13 +13346,13 @@
         <v>363</v>
       </c>
       <c r="B765" s="1">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="C765" s="1" t="s">
-        <v>364</v>
+        <v>516</v>
       </c>
       <c r="D765" s="3" t="s">
-        <v>35</v>
+        <v>405</v>
       </c>
     </row>
     <row r="766" spans="1:4" x14ac:dyDescent="0.45">
@@ -13357,13 +13360,13 @@
         <v>363</v>
       </c>
       <c r="B766" s="1">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="C766" s="1" t="s">
-        <v>517</v>
+        <v>364</v>
       </c>
       <c r="D766" s="3" t="s">
-        <v>395</v>
+        <v>35</v>
       </c>
     </row>
     <row r="767" spans="1:4" x14ac:dyDescent="0.45">
@@ -13374,7 +13377,7 @@
         <v>20</v>
       </c>
       <c r="C767" s="1" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
       <c r="D767" s="3" t="s">
         <v>395</v>
@@ -13385,13 +13388,13 @@
         <v>363</v>
       </c>
       <c r="B768" s="1">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="C768" s="1" t="s">
-        <v>366</v>
+        <v>518</v>
       </c>
       <c r="D768" s="3" t="s">
-        <v>27</v>
+        <v>395</v>
       </c>
     </row>
     <row r="769" spans="1:4" x14ac:dyDescent="0.45">
@@ -13399,13 +13402,13 @@
         <v>363</v>
       </c>
       <c r="B769" s="1">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="C769" s="1" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="D769" s="3" t="s">
-        <v>35</v>
+        <v>27</v>
       </c>
     </row>
     <row r="770" spans="1:4" x14ac:dyDescent="0.45">
@@ -13413,27 +13416,27 @@
         <v>363</v>
       </c>
       <c r="B770" s="1">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="C770" s="1" t="s">
-        <v>519</v>
+        <v>365</v>
       </c>
       <c r="D770" s="3" t="s">
-        <v>395</v>
+        <v>35</v>
       </c>
     </row>
     <row r="771" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A771" s="1" t="s">
-        <v>13</v>
+        <v>363</v>
       </c>
       <c r="B771" s="1">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="C771" s="1" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
       <c r="D771" s="3" t="s">
-        <v>402</v>
+        <v>395</v>
       </c>
     </row>
     <row r="772" spans="1:4" x14ac:dyDescent="0.45">
@@ -13441,13 +13444,13 @@
         <v>13</v>
       </c>
       <c r="B772" s="1">
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="C772" s="1" t="s">
-        <v>513</v>
+        <v>520</v>
       </c>
       <c r="D772" s="3" t="s">
-        <v>405</v>
+        <v>402</v>
       </c>
     </row>
     <row r="773" spans="1:4" x14ac:dyDescent="0.45">
@@ -13455,27 +13458,27 @@
         <v>13</v>
       </c>
       <c r="B773" s="1">
-        <v>20</v>
+        <v>60</v>
       </c>
       <c r="C773" s="1" t="s">
-        <v>509</v>
+        <v>513</v>
       </c>
       <c r="D773" s="3" t="s">
-        <v>395</v>
+        <v>405</v>
       </c>
     </row>
     <row r="774" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A774" s="1" t="s">
-        <v>367</v>
+        <v>13</v>
       </c>
       <c r="B774" s="1">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="C774" s="1" t="s">
-        <v>520</v>
+        <v>509</v>
       </c>
       <c r="D774" s="3" t="s">
-        <v>20</v>
+        <v>395</v>
       </c>
     </row>
     <row r="775" spans="1:4" x14ac:dyDescent="0.45">
@@ -13483,10 +13486,10 @@
         <v>367</v>
       </c>
       <c r="B775" s="1">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="C775" s="1" t="s">
-        <v>509</v>
+        <v>520</v>
       </c>
       <c r="D775" s="3" t="s">
         <v>20</v>
@@ -13497,10 +13500,10 @@
         <v>367</v>
       </c>
       <c r="B776" s="1">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="C776" s="1" t="s">
-        <v>112</v>
+        <v>509</v>
       </c>
       <c r="D776" s="3" t="s">
         <v>20</v>
@@ -13511,13 +13514,13 @@
         <v>367</v>
       </c>
       <c r="B777" s="1">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="C777" s="1" t="s">
-        <v>521</v>
+        <v>112</v>
       </c>
       <c r="D777" s="3" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
     <row r="778" spans="1:4" x14ac:dyDescent="0.45">
@@ -13525,13 +13528,13 @@
         <v>367</v>
       </c>
       <c r="B778" s="1">
-        <v>75</v>
+        <v>20</v>
       </c>
       <c r="C778" s="1" t="s">
-        <v>368</v>
+        <v>521</v>
       </c>
       <c r="D778" s="3" t="s">
-        <v>220</v>
+        <v>22</v>
       </c>
     </row>
     <row r="779" spans="1:4" x14ac:dyDescent="0.45">
@@ -13539,10 +13542,10 @@
         <v>367</v>
       </c>
       <c r="B779" s="1">
-        <v>20</v>
+        <v>75</v>
       </c>
       <c r="C779" s="1" t="s">
-        <v>522</v>
+        <v>368</v>
       </c>
       <c r="D779" s="3" t="s">
         <v>220</v>
@@ -13553,27 +13556,27 @@
         <v>367</v>
       </c>
       <c r="B780" s="1">
-        <v>60</v>
+        <v>20</v>
       </c>
       <c r="C780" s="1" t="s">
-        <v>369</v>
+        <v>522</v>
       </c>
       <c r="D780" s="3" t="s">
-        <v>213</v>
+        <v>220</v>
       </c>
     </row>
     <row r="781" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A781" s="1" t="s">
-        <v>370</v>
+        <v>367</v>
       </c>
       <c r="B781" s="1">
-        <v>100</v>
+        <v>60</v>
       </c>
       <c r="C781" s="1" t="s">
-        <v>513</v>
+        <v>369</v>
       </c>
       <c r="D781" s="3" t="s">
-        <v>22</v>
+        <v>213</v>
       </c>
     </row>
     <row r="782" spans="1:4" x14ac:dyDescent="0.45">
@@ -13581,24 +13584,24 @@
         <v>370</v>
       </c>
       <c r="B782" s="1">
-        <v>40</v>
+        <v>100</v>
       </c>
       <c r="C782" s="1" t="s">
-        <v>509</v>
+        <v>513</v>
       </c>
       <c r="D782" s="3" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
     </row>
     <row r="783" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A783" s="1" t="s">
-        <v>373</v>
+        <v>370</v>
       </c>
       <c r="B783" s="1">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="C783" s="1" t="s">
-        <v>23</v>
+        <v>509</v>
       </c>
       <c r="D783" s="3" t="s">
         <v>20</v>
@@ -13609,10 +13612,10 @@
         <v>373</v>
       </c>
       <c r="B784" s="1">
-        <v>75</v>
+        <v>50</v>
       </c>
       <c r="C784" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D784" s="3" t="s">
         <v>20</v>
@@ -13623,10 +13626,10 @@
         <v>373</v>
       </c>
       <c r="B785" s="1">
-        <v>30</v>
+        <v>75</v>
       </c>
       <c r="C785" s="1" t="s">
-        <v>33</v>
+        <v>24</v>
       </c>
       <c r="D785" s="3" t="s">
         <v>20</v>
@@ -13634,27 +13637,27 @@
     </row>
     <row r="786" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A786" s="1" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="B786" s="1">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="C786" s="1" t="s">
-        <v>520</v>
+        <v>33</v>
       </c>
       <c r="D786" s="3" t="s">
-        <v>402</v>
+        <v>20</v>
       </c>
     </row>
     <row r="787" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A787" s="1" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="B787" s="1">
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="C787" s="1" t="s">
-        <v>510</v>
+        <v>520</v>
       </c>
       <c r="D787" s="3" t="s">
         <v>402</v>
@@ -13665,27 +13668,27 @@
         <v>372</v>
       </c>
       <c r="B788" s="1">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="C788" s="1" t="s">
-        <v>523</v>
+        <v>510</v>
       </c>
       <c r="D788" s="3" t="s">
-        <v>395</v>
+        <v>402</v>
       </c>
     </row>
     <row r="789" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A789" s="1" t="s">
-        <v>374</v>
+        <v>372</v>
       </c>
       <c r="B789" s="1">
         <v>40</v>
       </c>
       <c r="C789" s="1" t="s">
-        <v>520</v>
+        <v>523</v>
       </c>
       <c r="D789" s="3" t="s">
-        <v>20</v>
+        <v>395</v>
       </c>
     </row>
     <row r="790" spans="1:4" x14ac:dyDescent="0.45">
@@ -13696,7 +13699,7 @@
         <v>40</v>
       </c>
       <c r="C790" s="1" t="s">
-        <v>523</v>
+        <v>520</v>
       </c>
       <c r="D790" s="3" t="s">
         <v>20</v>
@@ -13707,10 +13710,10 @@
         <v>374</v>
       </c>
       <c r="B791" s="1">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="C791" s="1" t="s">
-        <v>24</v>
+        <v>523</v>
       </c>
       <c r="D791" s="3" t="s">
         <v>20</v>
@@ -13721,13 +13724,13 @@
         <v>374</v>
       </c>
       <c r="B792" s="1">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="C792" s="1" t="s">
-        <v>33</v>
+        <v>24</v>
       </c>
       <c r="D792" s="3" t="s">
-        <v>35</v>
+        <v>20</v>
       </c>
     </row>
     <row r="793" spans="1:4" x14ac:dyDescent="0.45">
@@ -13735,10 +13738,10 @@
         <v>374</v>
       </c>
       <c r="B793" s="1">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="C793" s="1" t="s">
-        <v>524</v>
+        <v>33</v>
       </c>
       <c r="D793" s="3" t="s">
         <v>35</v>
@@ -13746,16 +13749,16 @@
     </row>
     <row r="794" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A794" s="1" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="B794" s="1">
-        <v>40</v>
+        <v>25</v>
       </c>
       <c r="C794" s="1" t="s">
-        <v>520</v>
+        <v>524</v>
       </c>
       <c r="D794" s="3" t="s">
-        <v>402</v>
+        <v>35</v>
       </c>
     </row>
     <row r="795" spans="1:4" x14ac:dyDescent="0.45">
@@ -13763,13 +13766,13 @@
         <v>375</v>
       </c>
       <c r="B795" s="1">
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="C795" s="1" t="s">
-        <v>33</v>
+        <v>520</v>
       </c>
       <c r="D795" s="3" t="s">
-        <v>35</v>
+        <v>402</v>
       </c>
     </row>
     <row r="796" spans="1:4" x14ac:dyDescent="0.45">
@@ -13777,13 +13780,13 @@
         <v>375</v>
       </c>
       <c r="B796" s="1">
-        <v>300</v>
+        <v>60</v>
       </c>
       <c r="C796" s="1" t="s">
-        <v>24</v>
+        <v>33</v>
       </c>
       <c r="D796" s="3" t="s">
-        <v>27</v>
+        <v>35</v>
       </c>
     </row>
     <row r="797" spans="1:4" x14ac:dyDescent="0.45">
@@ -13791,13 +13794,13 @@
         <v>375</v>
       </c>
       <c r="B797" s="1">
-        <v>80</v>
+        <v>300</v>
       </c>
       <c r="C797" s="1" t="s">
-        <v>525</v>
+        <v>24</v>
       </c>
       <c r="D797" s="3" t="s">
-        <v>405</v>
+        <v>27</v>
       </c>
     </row>
     <row r="798" spans="1:4" x14ac:dyDescent="0.45">
@@ -13805,13 +13808,13 @@
         <v>375</v>
       </c>
       <c r="B798" s="1">
-        <v>50</v>
+        <v>80</v>
       </c>
       <c r="C798" s="1" t="s">
-        <v>376</v>
+        <v>525</v>
       </c>
       <c r="D798" s="3" t="s">
-        <v>35</v>
+        <v>405</v>
       </c>
     </row>
     <row r="799" spans="1:4" x14ac:dyDescent="0.45">
@@ -13819,10 +13822,10 @@
         <v>375</v>
       </c>
       <c r="B799" s="1">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="C799" s="1" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="D799" s="3" t="s">
         <v>35</v>
@@ -13833,10 +13836,10 @@
         <v>375</v>
       </c>
       <c r="B800" s="1">
-        <v>175</v>
+        <v>60</v>
       </c>
       <c r="C800" s="1" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="D800" s="3" t="s">
         <v>35</v>
@@ -13847,13 +13850,13 @@
         <v>375</v>
       </c>
       <c r="B801" s="1">
-        <v>30</v>
+        <v>175</v>
       </c>
       <c r="C801" s="1" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="D801" s="3" t="s">
-        <v>218</v>
+        <v>35</v>
       </c>
     </row>
     <row r="802" spans="1:4" x14ac:dyDescent="0.45">
@@ -13861,27 +13864,27 @@
         <v>375</v>
       </c>
       <c r="B802" s="1">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="C802" s="1" t="s">
-        <v>526</v>
+        <v>379</v>
       </c>
       <c r="D802" s="3" t="s">
-        <v>403</v>
+        <v>218</v>
       </c>
     </row>
     <row r="803" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A803" s="1" t="s">
-        <v>380</v>
+        <v>375</v>
       </c>
       <c r="B803" s="1">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="C803" s="1" t="s">
-        <v>513</v>
+        <v>526</v>
       </c>
       <c r="D803" s="3" t="s">
-        <v>396</v>
+        <v>403</v>
       </c>
     </row>
     <row r="804" spans="1:4" x14ac:dyDescent="0.45">
@@ -13892,10 +13895,10 @@
         <v>20</v>
       </c>
       <c r="C804" s="1" t="s">
-        <v>510</v>
+        <v>513</v>
       </c>
       <c r="D804" s="3" t="s">
-        <v>20</v>
+        <v>396</v>
       </c>
     </row>
     <row r="805" spans="1:4" x14ac:dyDescent="0.45">
@@ -13903,10 +13906,10 @@
         <v>380</v>
       </c>
       <c r="B805" s="1">
-        <v>75</v>
+        <v>20</v>
       </c>
       <c r="C805" s="1" t="s">
-        <v>24</v>
+        <v>510</v>
       </c>
       <c r="D805" s="3" t="s">
         <v>20</v>
@@ -13920,10 +13923,10 @@
         <v>75</v>
       </c>
       <c r="C806" s="1" t="s">
-        <v>400</v>
+        <v>24</v>
       </c>
       <c r="D806" s="3" t="s">
-        <v>35</v>
+        <v>20</v>
       </c>
     </row>
     <row r="807" spans="1:4" x14ac:dyDescent="0.45">
@@ -13931,10 +13934,10 @@
         <v>380</v>
       </c>
       <c r="B807" s="1">
-        <v>30</v>
+        <v>75</v>
       </c>
       <c r="C807" s="1" t="s">
-        <v>33</v>
+        <v>400</v>
       </c>
       <c r="D807" s="3" t="s">
         <v>35</v>
@@ -13942,16 +13945,16 @@
     </row>
     <row r="808" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A808" s="1" t="s">
-        <v>382</v>
+        <v>380</v>
       </c>
       <c r="B808" s="1">
-        <v>75</v>
+        <v>30</v>
       </c>
       <c r="C808" s="1" t="s">
-        <v>381</v>
+        <v>33</v>
       </c>
       <c r="D808" s="3" t="s">
-        <v>20</v>
+        <v>35</v>
       </c>
     </row>
     <row r="809" spans="1:4" x14ac:dyDescent="0.45">
@@ -13959,13 +13962,13 @@
         <v>382</v>
       </c>
       <c r="B809" s="1">
-        <v>20</v>
+        <v>75</v>
       </c>
       <c r="C809" s="1" t="s">
-        <v>527</v>
+        <v>381</v>
       </c>
       <c r="D809" s="3" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
     <row r="810" spans="1:4" x14ac:dyDescent="0.45">
@@ -13973,27 +13976,27 @@
         <v>382</v>
       </c>
       <c r="B810" s="1">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="C810" s="1" t="s">
-        <v>528</v>
+        <v>527</v>
       </c>
       <c r="D810" s="3" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
     </row>
     <row r="811" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A811" s="1" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="B811" s="1">
         <v>40</v>
       </c>
       <c r="C811" s="1" t="s">
-        <v>513</v>
+        <v>528</v>
       </c>
       <c r="D811" s="3" t="s">
-        <v>405</v>
+        <v>20</v>
       </c>
     </row>
     <row r="812" spans="1:4" x14ac:dyDescent="0.45">
@@ -14001,13 +14004,13 @@
         <v>383</v>
       </c>
       <c r="B812" s="1">
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="C812" s="1" t="s">
-        <v>520</v>
+        <v>513</v>
       </c>
       <c r="D812" s="3" t="s">
-        <v>402</v>
+        <v>405</v>
       </c>
     </row>
     <row r="813" spans="1:4" x14ac:dyDescent="0.45">
@@ -14015,13 +14018,13 @@
         <v>383</v>
       </c>
       <c r="B813" s="1">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="C813" s="1" t="s">
-        <v>33</v>
+        <v>520</v>
       </c>
       <c r="D813" s="3" t="s">
-        <v>35</v>
+        <v>402</v>
       </c>
     </row>
     <row r="814" spans="1:4" x14ac:dyDescent="0.45">
@@ -14029,13 +14032,13 @@
         <v>383</v>
       </c>
       <c r="B814" s="1">
-        <v>75</v>
+        <v>30</v>
       </c>
       <c r="C814" s="1" t="s">
-        <v>24</v>
+        <v>33</v>
       </c>
       <c r="D814" s="3" t="s">
-        <v>27</v>
+        <v>35</v>
       </c>
     </row>
     <row r="815" spans="1:4" x14ac:dyDescent="0.45">
@@ -14043,13 +14046,13 @@
         <v>383</v>
       </c>
       <c r="B815" s="1">
-        <v>50</v>
+        <v>75</v>
       </c>
       <c r="C815" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D815" s="3" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="816" spans="1:4" x14ac:dyDescent="0.45">
@@ -14057,13 +14060,13 @@
         <v>383</v>
       </c>
       <c r="B816" s="1">
-        <v>20</v>
+        <v>50</v>
       </c>
       <c r="C816" s="1" t="s">
-        <v>509</v>
+        <v>23</v>
       </c>
       <c r="D816" s="3" t="s">
-        <v>395</v>
+        <v>26</v>
       </c>
     </row>
     <row r="817" spans="1:4" x14ac:dyDescent="0.45">
@@ -14071,13 +14074,13 @@
         <v>383</v>
       </c>
       <c r="B817" s="1">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="C817" s="1" t="s">
-        <v>384</v>
+        <v>509</v>
       </c>
       <c r="D817" s="3" t="s">
-        <v>401</v>
+        <v>395</v>
       </c>
     </row>
     <row r="818" spans="1:4" x14ac:dyDescent="0.45">
@@ -14085,47 +14088,61 @@
         <v>383</v>
       </c>
       <c r="B818" s="1">
-        <v>20</v>
+        <v>50</v>
       </c>
       <c r="C818" s="1" t="s">
+        <v>384</v>
+      </c>
+      <c r="D818" s="3" t="s">
+        <v>401</v>
+      </c>
+    </row>
+    <row r="819" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A819" s="1" t="s">
+        <v>383</v>
+      </c>
+      <c r="B819" s="1">
+        <v>20</v>
+      </c>
+      <c r="C819" s="1" t="s">
         <v>529</v>
       </c>
-      <c r="D818" s="3" t="s">
+      <c r="D819" s="3" t="s">
         <v>404</v>
-      </c>
-    </row>
-    <row r="820" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A820" s="1" t="s">
-        <v>410</v>
-      </c>
-      <c r="B820" s="1">
-        <f>SUM(B2:B818)</f>
-        <v>141643</v>
       </c>
     </row>
     <row r="821" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A821" s="1" t="s">
-        <v>17</v>
+        <v>410</v>
       </c>
       <c r="B821" s="1">
-        <v>20203</v>
+        <f>SUM(B2:B819)</f>
+        <v>141913</v>
       </c>
     </row>
     <row r="822" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A822" s="1" t="s">
-        <v>634</v>
+        <v>17</v>
       </c>
       <c r="B822" s="1">
-        <v>16353</v>
+        <v>20203</v>
       </c>
     </row>
     <row r="823" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A823" s="1" t="s">
+        <v>634</v>
+      </c>
+      <c r="B823" s="1">
+        <v>16353</v>
+      </c>
+    </row>
+    <row r="824" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A824" s="1" t="s">
         <v>635</v>
       </c>
-      <c r="B823" s="1">
-        <f>B820-B821-B822</f>
-        <v>105087</v>
+      <c r="B824" s="1">
+        <f>B821-B822-B823</f>
+        <v>105357</v>
       </c>
     </row>
   </sheetData>
@@ -19568,8 +19585,7 @@
         <v>307</v>
       </c>
       <c r="B392" s="1">
-        <f>1234+180</f>
-        <v>1414</v>
+        <v>1684</v>
       </c>
       <c r="C392" s="1" t="s">
         <v>611</v>
@@ -22348,11 +22364,11 @@
       </c>
       <c r="B593" s="1">
         <f>SUM(B2:B591)</f>
-        <v>141643</v>
+        <v>141913</v>
       </c>
       <c r="C593" s="1" t="str">
-        <f>"should be " &amp; 'New Gems (simplified per-rule)'!B820</f>
-        <v>should be 141643</v>
+        <f>"should be " &amp; 'New Gems (simplified per-rule)'!B821</f>
+        <v>should be 141913</v>
       </c>
     </row>
     <row r="594" spans="1:3" x14ac:dyDescent="0.45">
@@ -22377,11 +22393,11 @@
       </c>
       <c r="B596" s="1">
         <f>B593-B594-B595</f>
-        <v>105087</v>
+        <v>105357</v>
       </c>
       <c r="C596" s="1" t="str">
-        <f>"should be " &amp; 'New Gems (simplified per-rule)'!B823</f>
-        <v>should be 105087</v>
+        <f>"should be " &amp; 'New Gems (simplified per-rule)'!B824</f>
+        <v>should be 105357</v>
       </c>
     </row>
   </sheetData>

</xml_diff>